<commit_message>
Roll the listed spread names to November
TT's short name for the inter-product spread is "CL Nov26 - BZ Nov26
Inter-Product", confirmed from the platform. The crack follows the same
pattern as its October name, so "Nov26 HO-CL Crack" - that one is inferred
from the pattern rather than read off TT, and should be checked.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HHvxabz67VZkmriPMTpFvX
</commit_message>
<xml_diff>
--- a/TT_ZScore_Monitor.xlsx
+++ b/TT_ZScore_Monitor.xlsx
@@ -5465,7 +5465,7 @@
       </c>
       <c r="B86" s="259" t="inlineStr">
         <is>
-          <t>CL Oct26 - BZ Oct26 Inter-Product</t>
+          <t>CL Nov26 - BZ Nov26 Inter-Product</t>
         </is>
       </c>
       <c r="C86" s="235" t="inlineStr">
@@ -5487,7 +5487,7 @@
       </c>
       <c r="B87" s="259" t="inlineStr">
         <is>
-          <t>Oct26 HO-CL Crack</t>
+          <t>Nov26 HO-CL Crack</t>
         </is>
       </c>
       <c r="C87" s="235" t="inlineStr">

</xml_diff>